<commit_message>
docs(grants): update strategy, add technical whitepaper, and integrate strategic differentiators
</commit_message>
<xml_diff>
--- a/grants/SCORE Financial Projections Template.xlsx
+++ b/grants/SCORE Financial Projections Template.xlsx
@@ -34037,7 +34037,7 @@
       </c>
       <c r="O8" s="506" t="inlineStr">
         <is>
-          <t>Annual Totals</t>
+          <t>STRATEGIC DIFFERENTIATORS</t>
         </is>
       </c>
     </row>
@@ -34060,7 +34060,11 @@
       <c r="L9" s="151" t="n"/>
       <c r="M9" s="151" t="n"/>
       <c r="N9" s="151" t="n"/>
-      <c r="O9" s="152" t="n"/>
+      <c r="O9" s="152" t="inlineStr">
+        <is>
+          <t>Market Advantage: Filling gaps in fixed ALPR with mobile nodes.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="145" t="n"/>
@@ -34081,9 +34085,10 @@
       <c r="L10" s="154" t="n"/>
       <c r="M10" s="154" t="n"/>
       <c r="N10" s="154" t="n"/>
-      <c r="O10" s="60">
-        <f>SUM(C10:N10)</f>
-        <v/>
+      <c r="O10" s="60" t="inlineStr">
+        <is>
+          <t>Sustainability: Low overhead via community-volunteered hardware.</t>
+        </is>
       </c>
     </row>
     <row r="11">

</xml_diff>